<commit_message>
docs: report reduced performance duration averaged over ten decode steps
Keep the requested single-sheet 16-column layout. Duration is mean cumulative time per decode step for each operator name. Retain duration-weighted ratios and the skill calculation of per-call contributions before aggregation.

Co-authored-by: Codex <noreply@openai.com>

Signed-off-by: xiayehui <530885617@qq.com>
</commit_message>
<xml_diff>
--- a/reduced/performance/减层性能分析.xlsx
+++ b/reduced/performance/减层性能分析.xlsx
@@ -476,7 +476,7 @@
         <v>aclnnMatmul_MatMulV3Common_MatMulV3</v>
       </c>
       <c r="B2" s="1">
-        <v>9330.593</v>
+        <v>933.0593000000001</v>
       </c>
       <c r="C2" s="2">
         <v>0.5964426745438369</v>
@@ -526,7 +526,7 @@
         <v>aclnnInplaceCopy_CastAiCore_Cast</v>
       </c>
       <c r="B3" s="1">
-        <v>7767.641000000004</v>
+        <v>776.7641000000004</v>
       </c>
       <c r="C3" s="2">
         <v>0</v>
@@ -576,7 +576,7 @@
         <v>LightningIndexer</v>
       </c>
       <c r="B4" s="1">
-        <v>1899.544</v>
+        <v>189.95440000000002</v>
       </c>
       <c r="C4" s="2">
         <v>0.2689878986746293</v>
@@ -626,7 +626,7 @@
         <v>SparseFlashAttention</v>
       </c>
       <c r="B5" s="1">
-        <v>1476.69</v>
+        <v>147.669</v>
       </c>
       <c r="C5" s="2">
         <v>0.07367623536422675</v>
@@ -676,7 +676,7 @@
         <v>aclnnGroupedMatmulV5_GroupedMatmul_GroupedMatmul</v>
       </c>
       <c r="B6" s="1">
-        <v>1113.913</v>
+        <v>111.3913</v>
       </c>
       <c r="C6" s="2">
         <v>0.24772679733515998</v>
@@ -726,7 +726,7 @@
         <v>MoeDistributeCombineV3</v>
       </c>
       <c r="B7" s="1">
-        <v>541.265</v>
+        <v>54.1265</v>
       </c>
       <c r="C7" s="2">
         <v>0</v>
@@ -776,7 +776,7 @@
         <v>aclnnTransposeBatchMatMul_TransposeBatchMatMul_TransposeBatchMatMul</v>
       </c>
       <c r="B8" s="1">
-        <v>327.1899999999999</v>
+        <v>32.71899999999999</v>
       </c>
       <c r="C8" s="2">
         <v>0.09412117118493846</v>
@@ -826,7 +826,7 @@
         <v>_ihc_pre_stage2</v>
       </c>
       <c r="B9" s="1">
-        <v>316.38500000000005</v>
+        <v>31.638500000000004</v>
       </c>
       <c r="C9" s="2">
         <v>0</v>
@@ -876,7 +876,7 @@
         <v>MoeDistributeDispatchV3</v>
       </c>
       <c r="B10" s="1">
-        <v>303.418</v>
+        <v>30.3418</v>
       </c>
       <c r="C10" s="2">
         <v>0</v>
@@ -926,7 +926,7 @@
         <v>aclnnCat_ConcatD_ConcatD</v>
       </c>
       <c r="B11" s="1">
-        <v>284.13</v>
+        <v>28.413</v>
       </c>
       <c r="C11" s="2">
         <v>0</v>
@@ -976,7 +976,7 @@
         <v>RmsNorm</v>
       </c>
       <c r="B12" s="1">
-        <v>232.65900000000002</v>
+        <v>23.265900000000002</v>
       </c>
       <c r="C12" s="2">
         <v>0</v>
@@ -1026,7 +1026,7 @@
         <v>_ihc_pre_stage1</v>
       </c>
       <c r="B13" s="1">
-        <v>171.488</v>
+        <v>17.1488</v>
       </c>
       <c r="C13" s="2">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>aclnnAdd_AddAiCore_Add</v>
       </c>
       <c r="B14" s="1">
-        <v>168.4850000000001</v>
+        <v>16.84850000000001</v>
       </c>
       <c r="C14" s="2">
         <v>0</v>
@@ -1126,7 +1126,7 @@
         <v>aclnnMul_MulAiCore_Mul</v>
       </c>
       <c r="B15" s="1">
-        <v>165.76800000000006</v>
+        <v>16.576800000000006</v>
       </c>
       <c r="C15" s="2">
         <v>0</v>
@@ -1176,7 +1176,7 @@
         <v>_ihc_post_kernel</v>
       </c>
       <c r="B16" s="1">
-        <v>160.49599999999998</v>
+        <v>16.049599999999998</v>
       </c>
       <c r="C16" s="2">
         <v>0</v>
@@ -1226,7 +1226,7 @@
         <v>aclnnRemainderTensorScalar_FloorModAiCore_FloorMod</v>
       </c>
       <c r="B17" s="1">
-        <v>148.06099999999998</v>
+        <v>14.806099999999997</v>
       </c>
       <c r="C17" s="2">
         <v>0</v>
@@ -1276,7 +1276,7 @@
         <v>aclnnSoftmax_SoftmaxAiCore_SoftmaxV2</v>
       </c>
       <c r="B18" s="1">
-        <v>146.78300000000002</v>
+        <v>14.678300000000002</v>
       </c>
       <c r="C18" s="2">
         <v>0</v>
@@ -1326,7 +1326,7 @@
         <v>aclnnInplaceFillScalar_FillAiCore_Fill</v>
       </c>
       <c r="B19" s="1">
-        <v>136.62699999999998</v>
+        <v>13.662699999999997</v>
       </c>
       <c r="C19" s="2">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>aclnnSigmoid_SigmoidAiCore_Sigmoid</v>
       </c>
       <c r="B20" s="1">
-        <v>130.057</v>
+        <v>13.0057</v>
       </c>
       <c r="C20" s="2">
         <v>0</v>
@@ -1426,7 +1426,7 @@
         <v>aclnnBitwiseAndTensor_LogicalAndAiCore_LogicalAnd</v>
       </c>
       <c r="B21" s="1">
-        <v>124.52899999999993</v>
+        <v>12.452899999999993</v>
       </c>
       <c r="C21" s="2">
         <v>0</v>
@@ -1476,7 +1476,7 @@
         <v>aclnnLeScalar_LessEqualAiCore_LessEqual</v>
       </c>
       <c r="B22" s="1">
-        <v>118.77500000000002</v>
+        <v>11.877500000000001</v>
       </c>
       <c r="C22" s="2">
         <v>0</v>
@@ -1526,7 +1526,7 @@
         <v>aclnnEqScalar_EqualAiCore_Equal</v>
       </c>
       <c r="B23" s="1">
-        <v>118.21099999999998</v>
+        <v>11.821099999999998</v>
       </c>
       <c r="C23" s="2">
         <v>0</v>
@@ -1576,7 +1576,7 @@
         <v>SimThreadExponential</v>
       </c>
       <c r="B24" s="1">
-        <v>108.528</v>
+        <v>10.8528</v>
       </c>
       <c r="C24" s="2">
         <v>0</v>
@@ -1626,7 +1626,7 @@
         <v>_triton_rope_siso</v>
       </c>
       <c r="B25" s="1">
-        <v>107.47100000000002</v>
+        <v>10.747100000000001</v>
       </c>
       <c r="C25" s="2">
         <v>0</v>
@@ -1676,7 +1676,7 @@
         <v>SwiGlu</v>
       </c>
       <c r="B26" s="1">
-        <v>96.16299999999998</v>
+        <v>9.616299999999999</v>
       </c>
       <c r="C26" s="2">
         <v>0</v>
@@ -1726,7 +1726,7 @@
         <v>aclnnMuls_MulAiCore_Mul</v>
       </c>
       <c r="B27" s="1">
-        <v>89.767</v>
+        <v>8.9767</v>
       </c>
       <c r="C27" s="2">
         <v>0</v>
@@ -1776,7 +1776,7 @@
         <v>aclnnSWhere_SelectV2AiCore_SelectV2</v>
       </c>
       <c r="B28" s="1">
-        <v>86.348</v>
+        <v>8.6348</v>
       </c>
       <c r="C28" s="2">
         <v>0</v>
@@ -1826,7 +1826,7 @@
         <v>aclnnRotaryPositionEmbedding_RotaryPositionEmbedding_RotaryPositionEmbedding</v>
       </c>
       <c r="B29" s="1">
-        <v>86.04999999999998</v>
+        <v>8.604999999999999</v>
       </c>
       <c r="C29" s="2">
         <v>0</v>
@@ -1876,7 +1876,7 @@
         <v>aclnnClamp_ViewCopyAiCore_ViewCopy</v>
       </c>
       <c r="B30" s="1">
-        <v>84.58699999999997</v>
+        <v>8.458699999999997</v>
       </c>
       <c r="C30" s="2">
         <v>0</v>
@@ -1926,7 +1926,7 @@
         <v>aclnnDiv_RealDivAiCore_RealDiv</v>
       </c>
       <c r="B31" s="1">
-        <v>78.401</v>
+        <v>7.8401</v>
       </c>
       <c r="C31" s="2">
         <v>0</v>
@@ -1976,7 +1976,7 @@
         <v>aclnnArange_ArangeAiCore_Range</v>
       </c>
       <c r="B32" s="1">
-        <v>72.33300000000003</v>
+        <v>7.2333000000000025</v>
       </c>
       <c r="C32" s="2">
         <v>0</v>
@@ -2026,7 +2026,7 @@
         <v>aclnnIndexSelect_GatherV2AiCore_GatherV2</v>
       </c>
       <c r="B33" s="1">
-        <v>72.32799999999999</v>
+        <v>7.232799999999999</v>
       </c>
       <c r="C33" s="2">
         <v>0</v>
@@ -2076,7 +2076,7 @@
         <v>aclnnIndex_IndexAiCore_Index</v>
       </c>
       <c r="B34" s="1">
-        <v>71.351</v>
+        <v>7.1350999999999996</v>
       </c>
       <c r="C34" s="2">
         <v>0</v>
@@ -2126,7 +2126,7 @@
         <v>aclnnSub_SubAiCore_Sub</v>
       </c>
       <c r="B35" s="1">
-        <v>69.82400000000001</v>
+        <v>6.982400000000001</v>
       </c>
       <c r="C35" s="2">
         <v>0</v>
@@ -2176,7 +2176,7 @@
         <v>aclnnIndexSelect_SliceAiCore_Slice</v>
       </c>
       <c r="B36" s="1">
-        <v>69.25700000000003</v>
+        <v>6.9257000000000035</v>
       </c>
       <c r="C36" s="2">
         <v>0</v>
@@ -2226,7 +2226,7 @@
         <v>aclnnTransposeBatchMatMul_SliceAiCore_Slice</v>
       </c>
       <c r="B37" s="1">
-        <v>62.173</v>
+        <v>6.2173</v>
       </c>
       <c r="C37" s="2">
         <v>0</v>
@@ -2276,7 +2276,7 @@
         <v>KvRmsNormRopeCache</v>
       </c>
       <c r="B38" s="1">
-        <v>60.90600000000001</v>
+        <v>6.090600000000001</v>
       </c>
       <c r="C38" s="2">
         <v>0</v>
@@ -2326,7 +2326,7 @@
         <v>aclnnMean_ReduceMeanAiCore_ReduceMean</v>
       </c>
       <c r="B39" s="1">
-        <v>60.58500000000001</v>
+        <v>6.0585</v>
       </c>
       <c r="C39" s="2">
         <v>0</v>
@@ -2376,7 +2376,7 @@
         <v>aclnnLayerNormWithImplMode_LayerNormV4_LayerNormV4</v>
       </c>
       <c r="B40" s="1">
-        <v>60.139999999999986</v>
+        <v>6.0139999999999985</v>
       </c>
       <c r="C40" s="2">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>aclnnReduceSum_ReduceSumOpAiCore_ReduceSum</v>
       </c>
       <c r="B41" s="1">
-        <v>60.05799999999999</v>
+        <v>6.005799999999999</v>
       </c>
       <c r="C41" s="2">
         <v>0</v>
@@ -2476,7 +2476,7 @@
         <v>MoeGatingTopK</v>
       </c>
       <c r="B42" s="1">
-        <v>58.079000000000015</v>
+        <v>5.807900000000002</v>
       </c>
       <c r="C42" s="2">
         <v>0</v>
@@ -2526,7 +2526,7 @@
         <v>aclnnInplaceMul_MulAiCore_Mul</v>
       </c>
       <c r="B43" s="1">
-        <v>56.90699999999999</v>
+        <v>5.690699999999999</v>
       </c>
       <c r="C43" s="2">
         <v>0</v>
@@ -2576,7 +2576,7 @@
         <v>ScatterPaCache</v>
       </c>
       <c r="B44" s="1">
-        <v>56.302</v>
+        <v>5.6302</v>
       </c>
       <c r="C44" s="2">
         <v>0</v>
@@ -2626,7 +2626,7 @@
         <v>aclnnRepeat_TileAiCore_Tile</v>
       </c>
       <c r="B45" s="1">
-        <v>55.46900000000001</v>
+        <v>5.546900000000001</v>
       </c>
       <c r="C45" s="2">
         <v>0</v>
@@ -2676,7 +2676,7 @@
         <v>aclnnClamp_ClipByValueV2AiCore_ClipByValueV2</v>
       </c>
       <c r="B46" s="1">
-        <v>55.132</v>
+        <v>5.513199999999999</v>
       </c>
       <c r="C46" s="2">
         <v>0</v>
@@ -2726,7 +2726,7 @@
         <v>aclnnClamp_SliceAiCore_Slice</v>
       </c>
       <c r="B47" s="1">
-        <v>53.721999999999994</v>
+        <v>5.372199999999999</v>
       </c>
       <c r="C47" s="2">
         <v>0</v>
@@ -2776,7 +2776,7 @@
         <v>aclnnRotaryPositionEmbedding_SliceAiCore_Slice</v>
       </c>
       <c r="B48" s="1">
-        <v>52.796</v>
+        <v>5.2796</v>
       </c>
       <c r="C48" s="2">
         <v>0</v>
@@ -2826,7 +2826,7 @@
         <v>aclnnGtScalar_GreaterAiCore_Greater</v>
       </c>
       <c r="B49" s="1">
-        <v>49.36700000000001</v>
+        <v>4.936700000000001</v>
       </c>
       <c r="C49" s="2">
         <v>0</v>
@@ -2876,7 +2876,7 @@
         <v>aclnnClampMin_ClipByValueV2AiCore_ClipByValueV2</v>
       </c>
       <c r="B50" s="1">
-        <v>49.05899999999999</v>
+        <v>4.905899999999999</v>
       </c>
       <c r="C50" s="2">
         <v>0</v>
@@ -2926,7 +2926,7 @@
         <v>aclnnArgMax_ArgMaxV2AiCore_ArgMaxV2</v>
       </c>
       <c r="B51" s="1">
-        <v>46.849000000000004</v>
+        <v>4.684900000000001</v>
       </c>
       <c r="C51" s="2">
         <v>0</v>
@@ -2976,7 +2976,7 @@
         <v>aclnnForeachAddListV2_ForeachAddListV2_ForeachAddList</v>
       </c>
       <c r="B52" s="1">
-        <v>43.989</v>
+        <v>4.398899999999999</v>
       </c>
       <c r="C52" s="2">
         <v>0</v>
@@ -3026,7 +3026,7 @@
         <v>_compute_slot_mapping_kernel</v>
       </c>
       <c r="B53" s="1">
-        <v>41.187000000000005</v>
+        <v>4.1187000000000005</v>
       </c>
       <c r="C53" s="2">
         <v>0</v>
@@ -3076,7 +3076,7 @@
         <v>aclnnLog_LogAiCore_Log</v>
       </c>
       <c r="B54" s="1">
-        <v>39.553</v>
+        <v>3.9553</v>
       </c>
       <c r="C54" s="2">
         <v>0</v>
@@ -3126,7 +3126,7 @@
         <v>aclnnInplaceCopy_SliceAiCore_Slice</v>
       </c>
       <c r="B55" s="1">
-        <v>35.121</v>
+        <v>3.5121</v>
       </c>
       <c r="C55" s="2">
         <v>0</v>
@@ -3176,7 +3176,7 @@
         <v>aclnnEmbedding_GatherV2AiCore_GatherV2</v>
       </c>
       <c r="B56" s="1">
-        <v>34.482</v>
+        <v>3.4482</v>
       </c>
       <c r="C56" s="2">
         <v>0</v>
@@ -3226,7 +3226,7 @@
         <v>aclnnAdds_AddAiCore_Add</v>
       </c>
       <c r="B57" s="1">
-        <v>33.766</v>
+        <v>3.3766</v>
       </c>
       <c r="C57" s="2">
         <v>0</v>
@@ -3276,7 +3276,7 @@
         <v>aclnnPowTensorScalar_SquareAiCore_Square</v>
       </c>
       <c r="B58" s="1">
-        <v>32.473</v>
+        <v>3.2473</v>
       </c>
       <c r="C58" s="2">
         <v>0</v>
@@ -3326,7 +3326,7 @@
         <v>aclnnGeScalar_GreaterEqual_GreaterEqual</v>
       </c>
       <c r="B59" s="1">
-        <v>28.764999999999997</v>
+        <v>2.8764999999999996</v>
       </c>
       <c r="C59" s="2">
         <v>0</v>
@@ -3376,7 +3376,7 @@
         <v>aclnnLtScalar_LessAiCore_Less</v>
       </c>
       <c r="B60" s="1">
-        <v>27.696000000000005</v>
+        <v>2.7696000000000005</v>
       </c>
       <c r="C60" s="2">
         <v>0</v>
@@ -3426,7 +3426,7 @@
         <v>aclnnRsqrt_RsqrtAiCore_Rsqrt</v>
       </c>
       <c r="B61" s="1">
-        <v>27.508000000000003</v>
+        <v>2.7508000000000004</v>
       </c>
       <c r="C61" s="2">
         <v>0</v>
@@ -3476,7 +3476,7 @@
         <v>aclnnInplaceMaskedFillScalar_MaskedFillAiCore_MaskedFill</v>
       </c>
       <c r="B62" s="1">
-        <v>26.759</v>
+        <v>2.6759</v>
       </c>
       <c r="C62" s="2">
         <v>0</v>
@@ -3526,7 +3526,7 @@
         <v>aclnnBitwiseNot_LogicalNotAiCore_LogicalNot</v>
       </c>
       <c r="B63" s="1">
-        <v>25.348999999999997</v>
+        <v>2.5348999999999995</v>
       </c>
       <c r="C63" s="2">
         <v>0</v>
@@ -3576,7 +3576,7 @@
         <v>aclnnArgMax_CastAiCore_Cast</v>
       </c>
       <c r="B64" s="1">
-        <v>23.477999999999998</v>
+        <v>2.3478</v>
       </c>
       <c r="C64" s="2">
         <v>0</v>
@@ -3626,7 +3626,7 @@
         <v>aclnnSubs_SubAiCore_Sub</v>
       </c>
       <c r="B65" s="1">
-        <v>21.778000000000002</v>
+        <v>2.1778000000000004</v>
       </c>
       <c r="C65" s="2">
         <v>0</v>
@@ -3676,7 +3676,7 @@
         <v>aclnnSub_CastAiCore_Cast</v>
       </c>
       <c r="B66" s="1">
-        <v>16.199</v>
+        <v>1.6199000000000001</v>
       </c>
       <c r="C66" s="2">
         <v>0</v>
@@ -3726,7 +3726,7 @@
         <v>aclnnMuls_CastAiCore_Cast</v>
       </c>
       <c r="B67" s="1">
-        <v>15.990000000000002</v>
+        <v>1.5990000000000002</v>
       </c>
       <c r="C67" s="2">
         <v>0</v>
@@ -3776,7 +3776,7 @@
         <v>aclnnMul_CastAiCore_Cast</v>
       </c>
       <c r="B68" s="1">
-        <v>14.779</v>
+        <v>1.4779</v>
       </c>
       <c r="C68" s="2">
         <v>0</v>

</xml_diff>